<commit_message>
Refresh add-sectors documentation assets
</commit_message>
<xml_diff>
--- a/mario/test/supporting_files/add_sectors/add_sector_iot_master_filled.xlsx
+++ b/mario/test/supporting_files/add_sectors/add_sector_iot_master_filled.xlsx
@@ -3,19 +3,21 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-39180" yWindow="3920" windowWidth="24380" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-39460" yWindow="6760" windowWidth="31280" windowHeight="14000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Regions Clusters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sectors Clusters" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DB units" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Total outputs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Trades" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Exclusions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Tolerances" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="new_ind" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="new_ser" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="s2b_r1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="s2b_r2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="s2b_r3" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Uncertainties" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DB units" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Total outputs" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Trades" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Exclusions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tolerances" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -37,7 +39,9 @@
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -96,19 +100,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -186,9 +186,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -226,7 +226,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -260,6 +260,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -294,9 +295,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -474,80 +476,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="7.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="13.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="8" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="15.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="18.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="11.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="11" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="14.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="8.1640625" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="6.5" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="16.33203125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="19.83203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="12.1640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="11.33203125" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="6.5" bestFit="1" customWidth="1" min="10" max="10"/>
     <col width="5.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="10.1640625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Inventory sheet</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Final consumption</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Consumption category</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Parent Sector</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Leave empty</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Add or Split</t>
         </is>
@@ -556,38 +557,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GLOBAL</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>New industry</t>
+          <t>s2b</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>new_ind</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
+          <t>s2b_r1</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Final demand</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>s2</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -599,38 +589,69 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Reg1</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New services</t>
+          <t>s2b</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>new_ser</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
+          <t>s2b_r2</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Final demand</t>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>r3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>s2b</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>s2b_r3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Split</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -640,51 +661,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.1640625" customWidth="1" min="2" max="2"/>
+    <col width="10.83203125" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Sector_from</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Region_from</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Region_to</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Item type</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>DB Item</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>DB Region</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Change type</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -695,33 +711,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>GLOBAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Reg2</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Sector_from</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Sector_to</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -730,7 +742,53 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>tol_Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1e-05</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1e-05</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -742,33 +800,82 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>GLOBAL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>r1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Services</t>
+          <t>r2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>r3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>s1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>s3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>s4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -778,169 +885,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="17" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="10.83203125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="6.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="17" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.83203125" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Item type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>DB Item</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Factor of production</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Taxes</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Factor of production</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Wages</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Factor of production</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Capital</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Satellite account</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Employment</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1000 p</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Satellite account</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CO2</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>kg</t>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>DB Region</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Change type</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -950,103 +950,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="11.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="6.5" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="10.1640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="6" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="9.6640625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="5.6640625" bestFit="1" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Item type</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>DB Item</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>DB Region</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Change type</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>New industry</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-      <c r="C2">
-        <f>0.05*53115504</f>
-        <v/>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>MARIO doc</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>New industry</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Reg2</t>
-        </is>
-      </c>
-      <c r="C3" s="5">
-        <f>0.05*1195683</f>
-        <v/>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MARIO doc</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1056,119 +1011,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="11.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="11" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="9" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="8" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="9.5" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="5.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sector_from</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Region_from</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Region_to</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Item type</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>DB Item</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>DB Region</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Change type</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>New industry</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Reg2</t>
-        </is>
-      </c>
-      <c r="D2" s="5">
-        <f>0.05*288442</f>
-        <v/>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MARIO doc</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>New industry</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Reg2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Reg1</t>
-        </is>
-      </c>
-      <c r="D3">
-        <f>0.05*437620</f>
-        <v/>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>M EUR</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MARIO doc</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1178,32 +1072,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
-  <cols>
-    <col width="13.5" customWidth="1" min="1" max="1"/>
-    <col width="12.1640625" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sector_from</t>
+          <t>Inventory data categories</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Sector_to</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
+          <t>New uncertainty values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>certain</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>original s specific, r cluster</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>original s specific_no parent, r cluster</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>original s cluster, r specific</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>original s cluster_no parent, r specific</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>original s cluster, r cluster</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>original s cluster_no parent, r cluster</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>disag s specific, r cluster</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>disag s cluster, r specific</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>disag s cluster_no parent, r specific</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>disag s cluster, r cluster</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>disag s specific_no parent, r cluster</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>disag s cluster_no parent, r cluster</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>no info</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>forced zero</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.005</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1213,39 +1248,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>tol_Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>values</t>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>unit</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>delta</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>s1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>eps</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>s2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>s2b</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>s3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>s4</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Factor of production</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Satellite account</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1259,51 +1391,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.5" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Item type</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>DB Item</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>DB Region</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Change type</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>